<commit_message>
fixing more unit business
</commit_message>
<xml_diff>
--- a/data/raw/51301-2026-02-medicaid.xlsx
+++ b/data/raw/51301-2026-02-medicaid.xlsx
@@ -632,51 +632,51 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -774,6 +774,10 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1122,13 +1126,13 @@
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
       <c r="L2" s="3"/>
-      <c r="M2" s="92" t="s">
+      <c r="M2" s="87" t="s">
         <v>35</v>
       </c>
-      <c r="N2" s="93"/>
-      <c r="O2" s="93"/>
-      <c r="P2" s="93"/>
-      <c r="Q2" s="93"/>
+      <c r="N2" s="88"/>
+      <c r="O2" s="88"/>
+      <c r="P2" s="88"/>
+      <c r="Q2" s="88"/>
       <c r="R2" s="4"/>
       <c r="V2" s="36"/>
       <c r="W2" s="36"/>
@@ -1205,16 +1209,16 @@
       <c r="X5" s="36"/>
     </row>
     <row r="6" spans="1:24" ht="17.600000000000001" x14ac:dyDescent="0.4">
-      <c r="A6" s="94" t="s">
+      <c r="A6" s="89" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="94"/>
-      <c r="C6" s="94"/>
-      <c r="D6" s="94"/>
-      <c r="E6" s="94"/>
-      <c r="F6" s="94"/>
-      <c r="G6" s="94"/>
-      <c r="H6" s="94"/>
+      <c r="B6" s="89"/>
+      <c r="C6" s="89"/>
+      <c r="D6" s="89"/>
+      <c r="E6" s="89"/>
+      <c r="F6" s="89"/>
+      <c r="G6" s="89"/>
+      <c r="H6" s="89"/>
       <c r="I6" s="42"/>
       <c r="J6" s="42"/>
       <c r="K6" s="42"/>
@@ -1246,10 +1250,10 @@
       <c r="M7" s="11"/>
       <c r="N7" s="11"/>
       <c r="O7" s="8"/>
-      <c r="P7" s="95" t="s">
+      <c r="P7" s="90" t="s">
         <v>36</v>
       </c>
-      <c r="Q7" s="95" t="s">
+      <c r="Q7" s="90" t="s">
         <v>37</v>
       </c>
       <c r="R7" s="4"/>
@@ -1295,8 +1299,8 @@
       <c r="O8" s="54">
         <v>2036</v>
       </c>
-      <c r="P8" s="96"/>
-      <c r="Q8" s="96"/>
+      <c r="P8" s="91"/>
+      <c r="Q8" s="91"/>
     </row>
     <row r="9" spans="1:24" ht="7.2" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="15"/>
@@ -1318,11 +1322,11 @@
       <c r="Q9" s="45"/>
     </row>
     <row r="10" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="86" t="s">
+      <c r="A10" s="82" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="86"/>
-      <c r="C10" s="86"/>
+      <c r="B10" s="82"/>
+      <c r="C10" s="82"/>
       <c r="D10" s="57"/>
       <c r="E10" s="57"/>
       <c r="F10" s="57"/>
@@ -1345,11 +1349,11 @@
       <c r="T10" s="7"/>
     </row>
     <row r="11" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="87" t="s">
+      <c r="A11" s="95" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="87"/>
-      <c r="C11" s="87"/>
+      <c r="B11" s="95"/>
+      <c r="C11" s="95"/>
       <c r="D11" s="57"/>
       <c r="E11" s="57"/>
       <c r="F11" s="57"/>
@@ -1390,11 +1394,11 @@
       <c r="T12" s="7"/>
     </row>
     <row r="13" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="86" t="s">
+      <c r="A13" s="82" t="s">
         <v>31</v>
       </c>
-      <c r="B13" s="86"/>
-      <c r="C13" s="86"/>
+      <c r="B13" s="82"/>
+      <c r="C13" s="82"/>
       <c r="D13" s="70">
         <v>668</v>
       </c>
@@ -1464,11 +1468,11 @@
       <c r="T14" s="7"/>
     </row>
     <row r="15" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="86" t="s">
+      <c r="A15" s="82" t="s">
         <v>5</v>
       </c>
-      <c r="B15" s="86"/>
-      <c r="C15" s="86"/>
+      <c r="B15" s="82"/>
+      <c r="C15" s="82"/>
       <c r="D15" s="75"/>
       <c r="E15" s="75"/>
       <c r="F15" s="75"/>
@@ -1488,10 +1492,10 @@
       <c r="T15" s="7"/>
     </row>
     <row r="16" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="82" t="s">
+      <c r="A16" s="93" t="s">
         <v>6</v>
       </c>
-      <c r="B16" s="82"/>
+      <c r="B16" s="93"/>
       <c r="C16" s="56"/>
       <c r="D16" s="61"/>
       <c r="E16" s="61"/>
@@ -1513,10 +1517,10 @@
     </row>
     <row r="17" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="56"/>
-      <c r="B17" s="84" t="s">
+      <c r="B17" s="83" t="s">
         <v>7</v>
       </c>
-      <c r="C17" s="84"/>
+      <c r="C17" s="83"/>
       <c r="D17" s="61"/>
       <c r="E17" s="61"/>
       <c r="F17" s="61"/>
@@ -1537,10 +1541,10 @@
     </row>
     <row r="18" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="60"/>
-      <c r="B18" s="85" t="s">
+      <c r="B18" s="94" t="s">
         <v>8</v>
       </c>
-      <c r="C18" s="85"/>
+      <c r="C18" s="94"/>
       <c r="D18" s="70">
         <v>142</v>
       </c>
@@ -1590,10 +1594,10 @@
     </row>
     <row r="19" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="56"/>
-      <c r="B19" s="85" t="s">
+      <c r="B19" s="94" t="s">
         <v>9</v>
       </c>
-      <c r="C19" s="85"/>
+      <c r="C19" s="94"/>
       <c r="D19" s="70">
         <v>295</v>
       </c>
@@ -1642,10 +1646,10 @@
     </row>
     <row r="20" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="56"/>
-      <c r="B20" s="85" t="s">
+      <c r="B20" s="94" t="s">
         <v>10</v>
       </c>
-      <c r="C20" s="85"/>
+      <c r="C20" s="94"/>
       <c r="D20" s="70">
         <v>16</v>
       </c>
@@ -1694,10 +1698,10 @@
     </row>
     <row r="21" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="56"/>
-      <c r="B21" s="84" t="s">
+      <c r="B21" s="83" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="84"/>
+      <c r="C21" s="83"/>
       <c r="D21" s="61"/>
       <c r="E21" s="61"/>
       <c r="F21" s="61"/>
@@ -1718,10 +1722,10 @@
     </row>
     <row r="22" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="56"/>
-      <c r="B22" s="85" t="s">
+      <c r="B22" s="94" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="85"/>
+      <c r="C22" s="94"/>
       <c r="D22" s="70">
         <v>64</v>
       </c>
@@ -1771,10 +1775,10 @@
     </row>
     <row r="23" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="56"/>
-      <c r="B23" s="85" t="s">
+      <c r="B23" s="94" t="s">
         <v>26</v>
       </c>
-      <c r="C23" s="85"/>
+      <c r="C23" s="94"/>
       <c r="D23" s="72">
         <v>110</v>
       </c>
@@ -1895,11 +1899,11 @@
       <c r="T25" s="7"/>
     </row>
     <row r="26" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="82" t="s">
+      <c r="A26" s="93" t="s">
         <v>13</v>
       </c>
-      <c r="B26" s="82"/>
-      <c r="C26" s="82"/>
+      <c r="B26" s="93"/>
+      <c r="C26" s="93"/>
       <c r="D26" s="70">
         <v>8</v>
       </c>
@@ -1947,11 +1951,11 @@
       <c r="T26" s="7"/>
     </row>
     <row r="27" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="82" t="s">
+      <c r="A27" s="93" t="s">
         <v>14</v>
       </c>
-      <c r="B27" s="82"/>
-      <c r="C27" s="82"/>
+      <c r="B27" s="93"/>
+      <c r="C27" s="93"/>
       <c r="D27" s="70">
         <v>7</v>
       </c>
@@ -1999,11 +2003,11 @@
       <c r="T27" s="7"/>
     </row>
     <row r="28" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="82" t="s">
+      <c r="A28" s="93" t="s">
         <v>15</v>
       </c>
-      <c r="B28" s="82"/>
-      <c r="C28" s="82"/>
+      <c r="B28" s="93"/>
+      <c r="C28" s="93"/>
       <c r="D28" s="70">
         <v>27</v>
       </c>
@@ -2096,11 +2100,11 @@
       <c r="T30" s="7"/>
     </row>
     <row r="31" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="83" t="s">
+      <c r="A31" s="97" t="s">
         <v>16</v>
       </c>
-      <c r="B31" s="83"/>
-      <c r="C31" s="83"/>
+      <c r="B31" s="97"/>
+      <c r="C31" s="97"/>
       <c r="D31" s="61"/>
       <c r="E31" s="61"/>
       <c r="F31" s="61"/>
@@ -2142,13 +2146,13 @@
       <c r="T32" s="7"/>
     </row>
     <row r="33" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="86" t="s">
+      <c r="A33" s="82" t="s">
         <v>43</v>
       </c>
-      <c r="B33" s="86"/>
-      <c r="C33" s="86"/>
-      <c r="D33" s="86"/>
-      <c r="E33" s="86"/>
+      <c r="B33" s="82"/>
+      <c r="C33" s="82"/>
+      <c r="D33" s="82"/>
+      <c r="E33" s="82"/>
       <c r="F33" s="61"/>
       <c r="G33" s="61"/>
       <c r="H33" s="61"/>
@@ -2166,10 +2170,10 @@
       <c r="T33" s="7"/>
     </row>
     <row r="34" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="88" t="s">
+      <c r="A34" s="96" t="s">
         <v>17</v>
       </c>
-      <c r="B34" s="88"/>
+      <c r="B34" s="96"/>
       <c r="C34" s="56"/>
       <c r="D34" s="70">
         <v>125</v>
@@ -2218,11 +2222,11 @@
       <c r="T34" s="7"/>
     </row>
     <row r="35" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="84" t="s">
+      <c r="A35" s="83" t="s">
         <v>18</v>
       </c>
-      <c r="B35" s="84"/>
-      <c r="C35" s="84"/>
+      <c r="B35" s="83"/>
+      <c r="C35" s="83"/>
       <c r="D35" s="70">
         <v>191</v>
       </c>
@@ -2270,10 +2274,10 @@
       <c r="T35" s="7"/>
     </row>
     <row r="36" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="84" t="s">
+      <c r="A36" s="83" t="s">
         <v>19</v>
       </c>
-      <c r="B36" s="84"/>
+      <c r="B36" s="83"/>
       <c r="C36" s="56"/>
       <c r="D36" s="70">
         <v>85</v>
@@ -2322,11 +2326,11 @@
       <c r="T36" s="7"/>
     </row>
     <row r="37" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="84" t="s">
+      <c r="A37" s="83" t="s">
         <v>42</v>
       </c>
-      <c r="B37" s="84"/>
-      <c r="C37" s="84"/>
+      <c r="B37" s="83"/>
+      <c r="C37" s="83"/>
       <c r="D37" s="70">
         <v>83</v>
       </c>
@@ -2374,11 +2378,11 @@
       <c r="T37" s="7"/>
     </row>
     <row r="38" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="84" t="s">
+      <c r="A38" s="83" t="s">
         <v>41</v>
       </c>
-      <c r="B38" s="84"/>
-      <c r="C38" s="84"/>
+      <c r="B38" s="83"/>
+      <c r="C38" s="83"/>
       <c r="D38" s="72">
         <v>144</v>
       </c>
@@ -2499,13 +2503,13 @@
       <c r="T40" s="7"/>
     </row>
     <row r="41" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="86" t="s">
+      <c r="A41" s="82" t="s">
         <v>27</v>
       </c>
-      <c r="B41" s="86"/>
-      <c r="C41" s="86"/>
-      <c r="D41" s="86"/>
-      <c r="E41" s="86"/>
+      <c r="B41" s="82"/>
+      <c r="C41" s="82"/>
+      <c r="D41" s="82"/>
+      <c r="E41" s="82"/>
       <c r="F41" s="61"/>
       <c r="G41" s="61"/>
       <c r="H41" s="61"/>
@@ -2523,10 +2527,10 @@
       <c r="T41" s="7"/>
     </row>
     <row r="42" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="84" t="s">
+      <c r="A42" s="83" t="s">
         <v>17</v>
       </c>
-      <c r="B42" s="84"/>
+      <c r="B42" s="83"/>
       <c r="C42" s="56"/>
       <c r="D42" s="70">
         <v>8</v>
@@ -2585,11 +2589,11 @@
       <c r="AD42" s="51"/>
     </row>
     <row r="43" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="84" t="s">
+      <c r="A43" s="83" t="s">
         <v>18</v>
       </c>
-      <c r="B43" s="84"/>
-      <c r="C43" s="84"/>
+      <c r="B43" s="83"/>
+      <c r="C43" s="83"/>
       <c r="D43" s="70">
         <v>9</v>
       </c>
@@ -2647,10 +2651,10 @@
       <c r="AD43" s="51"/>
     </row>
     <row r="44" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="84" t="s">
+      <c r="A44" s="83" t="s">
         <v>19</v>
       </c>
-      <c r="B44" s="84"/>
+      <c r="B44" s="83"/>
       <c r="C44" s="56"/>
       <c r="D44" s="70">
         <v>31</v>
@@ -2709,11 +2713,11 @@
       <c r="AD44" s="51"/>
     </row>
     <row r="45" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="84" t="s">
+      <c r="A45" s="83" t="s">
         <v>42</v>
       </c>
-      <c r="B45" s="84"/>
-      <c r="C45" s="84"/>
+      <c r="B45" s="83"/>
+      <c r="C45" s="83"/>
       <c r="D45" s="70">
         <v>17</v>
       </c>
@@ -2771,11 +2775,11 @@
       <c r="AD45" s="51"/>
     </row>
     <row r="46" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="84" t="s">
+      <c r="A46" s="83" t="s">
         <v>41</v>
       </c>
-      <c r="B46" s="84"/>
-      <c r="C46" s="84"/>
+      <c r="B46" s="83"/>
+      <c r="C46" s="83"/>
       <c r="D46" s="72">
         <v>17</v>
       </c>
@@ -2938,11 +2942,11 @@
       <c r="T49" s="7"/>
     </row>
     <row r="50" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="86" t="s">
+      <c r="A50" s="82" t="s">
         <v>22</v>
       </c>
-      <c r="B50" s="86"/>
-      <c r="C50" s="86"/>
+      <c r="B50" s="82"/>
+      <c r="C50" s="82"/>
       <c r="D50" s="66"/>
       <c r="E50" s="66"/>
       <c r="F50" s="66"/>
@@ -2972,11 +2976,11 @@
       <c r="AD50" s="46"/>
     </row>
     <row r="51" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="84" t="s">
+      <c r="A51" s="83" t="s">
         <v>28</v>
       </c>
-      <c r="B51" s="84"/>
-      <c r="C51" s="84"/>
+      <c r="B51" s="83"/>
+      <c r="C51" s="83"/>
       <c r="D51" s="70">
         <v>98</v>
       </c>
@@ -3066,13 +3070,13 @@
       <c r="AD52" s="46"/>
     </row>
     <row r="53" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="86" t="s">
+      <c r="A53" s="82" t="s">
         <v>39</v>
       </c>
-      <c r="B53" s="86"/>
-      <c r="C53" s="86"/>
-      <c r="D53" s="86"/>
-      <c r="E53" s="86"/>
+      <c r="B53" s="82"/>
+      <c r="C53" s="82"/>
+      <c r="D53" s="82"/>
+      <c r="E53" s="82"/>
       <c r="F53" s="66"/>
       <c r="G53" s="66"/>
       <c r="H53" s="66"/>
@@ -3304,11 +3308,11 @@
       <c r="T57" s="7"/>
     </row>
     <row r="58" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A58" s="84" t="s">
+      <c r="A58" s="83" t="s">
         <v>41</v>
       </c>
-      <c r="B58" s="84"/>
-      <c r="C58" s="84"/>
+      <c r="B58" s="83"/>
+      <c r="C58" s="83"/>
       <c r="D58" s="70">
         <v>8670</v>
       </c>
@@ -3444,49 +3448,49 @@
       <c r="A63" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B63" s="97" t="s">
+      <c r="B63" s="92" t="s">
         <v>40</v>
       </c>
-      <c r="C63" s="97"/>
-      <c r="D63" s="97"/>
-      <c r="E63" s="97"/>
-      <c r="F63" s="97"/>
-      <c r="G63" s="97"/>
-      <c r="H63" s="97"/>
-      <c r="I63" s="97"/>
-      <c r="J63" s="97"/>
-      <c r="K63" s="97"/>
-      <c r="L63" s="97"/>
-      <c r="M63" s="97"/>
-      <c r="N63" s="97"/>
-      <c r="O63" s="97"/>
-      <c r="P63" s="97"/>
-      <c r="Q63" s="97"/>
+      <c r="C63" s="92"/>
+      <c r="D63" s="92"/>
+      <c r="E63" s="92"/>
+      <c r="F63" s="92"/>
+      <c r="G63" s="92"/>
+      <c r="H63" s="92"/>
+      <c r="I63" s="92"/>
+      <c r="J63" s="92"/>
+      <c r="K63" s="92"/>
+      <c r="L63" s="92"/>
+      <c r="M63" s="92"/>
+      <c r="N63" s="92"/>
+      <c r="O63" s="92"/>
+      <c r="P63" s="92"/>
+      <c r="Q63" s="92"/>
       <c r="R63" s="47"/>
-      <c r="S63" s="91"/>
-      <c r="T63" s="91"/>
-      <c r="U63" s="91"/>
-      <c r="V63" s="91"/>
-      <c r="W63" s="91"/>
+      <c r="S63" s="86"/>
+      <c r="T63" s="86"/>
+      <c r="U63" s="86"/>
+      <c r="V63" s="86"/>
+      <c r="W63" s="86"/>
     </row>
     <row r="64" spans="1:30" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="9"/>
-      <c r="B64" s="97"/>
-      <c r="C64" s="97"/>
-      <c r="D64" s="97"/>
-      <c r="E64" s="97"/>
-      <c r="F64" s="97"/>
-      <c r="G64" s="97"/>
-      <c r="H64" s="97"/>
-      <c r="I64" s="97"/>
-      <c r="J64" s="97"/>
-      <c r="K64" s="97"/>
-      <c r="L64" s="97"/>
-      <c r="M64" s="97"/>
-      <c r="N64" s="97"/>
-      <c r="O64" s="97"/>
-      <c r="P64" s="97"/>
-      <c r="Q64" s="97"/>
+      <c r="B64" s="92"/>
+      <c r="C64" s="92"/>
+      <c r="D64" s="92"/>
+      <c r="E64" s="92"/>
+      <c r="F64" s="92"/>
+      <c r="G64" s="92"/>
+      <c r="H64" s="92"/>
+      <c r="I64" s="92"/>
+      <c r="J64" s="92"/>
+      <c r="K64" s="92"/>
+      <c r="L64" s="92"/>
+      <c r="M64" s="92"/>
+      <c r="N64" s="92"/>
+      <c r="O64" s="92"/>
+      <c r="P64" s="92"/>
+      <c r="Q64" s="92"/>
       <c r="R64" s="47"/>
       <c r="S64" s="47"/>
     </row>
@@ -3494,51 +3498,51 @@
       <c r="A65" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="B65" s="90" t="s">
+      <c r="B65" s="85" t="s">
         <v>34</v>
       </c>
-      <c r="C65" s="90"/>
-      <c r="D65" s="90"/>
-      <c r="E65" s="90"/>
-      <c r="F65" s="90"/>
-      <c r="G65" s="90"/>
-      <c r="H65" s="90"/>
-      <c r="I65" s="90"/>
-      <c r="J65" s="90"/>
-      <c r="K65" s="90"/>
-      <c r="L65" s="90"/>
-      <c r="M65" s="90"/>
-      <c r="N65" s="90"/>
-      <c r="O65" s="90"/>
-      <c r="P65" s="90"/>
-      <c r="Q65" s="90"/>
+      <c r="C65" s="85"/>
+      <c r="D65" s="85"/>
+      <c r="E65" s="85"/>
+      <c r="F65" s="85"/>
+      <c r="G65" s="85"/>
+      <c r="H65" s="85"/>
+      <c r="I65" s="85"/>
+      <c r="J65" s="85"/>
+      <c r="K65" s="85"/>
+      <c r="L65" s="85"/>
+      <c r="M65" s="85"/>
+      <c r="N65" s="85"/>
+      <c r="O65" s="85"/>
+      <c r="P65" s="85"/>
+      <c r="Q65" s="85"/>
       <c r="R65" s="47"/>
-      <c r="S65" s="89"/>
-      <c r="T65" s="89"/>
-      <c r="U65" s="89"/>
-      <c r="V65" s="89"/>
-      <c r="W65" s="89"/>
-      <c r="X65" s="89"/>
-      <c r="Y65" s="89"/>
+      <c r="S65" s="84"/>
+      <c r="T65" s="84"/>
+      <c r="U65" s="84"/>
+      <c r="V65" s="84"/>
+      <c r="W65" s="84"/>
+      <c r="X65" s="84"/>
+      <c r="Y65" s="84"/>
     </row>
     <row r="66" spans="1:25" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="9"/>
-      <c r="B66" s="90"/>
-      <c r="C66" s="90"/>
-      <c r="D66" s="90"/>
-      <c r="E66" s="90"/>
-      <c r="F66" s="90"/>
-      <c r="G66" s="90"/>
-      <c r="H66" s="90"/>
-      <c r="I66" s="90"/>
-      <c r="J66" s="90"/>
-      <c r="K66" s="90"/>
-      <c r="L66" s="90"/>
-      <c r="M66" s="90"/>
-      <c r="N66" s="90"/>
-      <c r="O66" s="90"/>
-      <c r="P66" s="90"/>
-      <c r="Q66" s="90"/>
+      <c r="B66" s="85"/>
+      <c r="C66" s="85"/>
+      <c r="D66" s="85"/>
+      <c r="E66" s="85"/>
+      <c r="F66" s="85"/>
+      <c r="G66" s="85"/>
+      <c r="H66" s="85"/>
+      <c r="I66" s="85"/>
+      <c r="J66" s="85"/>
+      <c r="K66" s="85"/>
+      <c r="L66" s="85"/>
+      <c r="M66" s="85"/>
+      <c r="N66" s="85"/>
+      <c r="O66" s="85"/>
+      <c r="P66" s="85"/>
+      <c r="Q66" s="85"/>
       <c r="R66" s="47"/>
       <c r="S66" s="47"/>
     </row>
@@ -3546,46 +3550,46 @@
       <c r="A67" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="B67" s="90" t="s">
+      <c r="B67" s="85" t="s">
         <v>38</v>
       </c>
-      <c r="C67" s="90"/>
-      <c r="D67" s="90"/>
-      <c r="E67" s="90"/>
-      <c r="F67" s="90"/>
-      <c r="G67" s="90"/>
-      <c r="H67" s="90"/>
-      <c r="I67" s="90"/>
-      <c r="J67" s="90"/>
-      <c r="K67" s="90"/>
-      <c r="L67" s="90"/>
-      <c r="M67" s="90"/>
-      <c r="N67" s="90"/>
-      <c r="O67" s="90"/>
-      <c r="P67" s="90"/>
-      <c r="Q67" s="90"/>
+      <c r="C67" s="85"/>
+      <c r="D67" s="85"/>
+      <c r="E67" s="85"/>
+      <c r="F67" s="85"/>
+      <c r="G67" s="85"/>
+      <c r="H67" s="85"/>
+      <c r="I67" s="85"/>
+      <c r="J67" s="85"/>
+      <c r="K67" s="85"/>
+      <c r="L67" s="85"/>
+      <c r="M67" s="85"/>
+      <c r="N67" s="85"/>
+      <c r="O67" s="85"/>
+      <c r="P67" s="85"/>
+      <c r="Q67" s="85"/>
       <c r="R67" s="7"/>
       <c r="S67" s="4"/>
       <c r="T67" s="7"/>
     </row>
     <row r="68" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A68" s="8"/>
-      <c r="B68" s="90"/>
-      <c r="C68" s="90"/>
-      <c r="D68" s="90"/>
-      <c r="E68" s="90"/>
-      <c r="F68" s="90"/>
-      <c r="G68" s="90"/>
-      <c r="H68" s="90"/>
-      <c r="I68" s="90"/>
-      <c r="J68" s="90"/>
-      <c r="K68" s="90"/>
-      <c r="L68" s="90"/>
-      <c r="M68" s="90"/>
-      <c r="N68" s="90"/>
-      <c r="O68" s="90"/>
-      <c r="P68" s="90"/>
-      <c r="Q68" s="90"/>
+      <c r="B68" s="85"/>
+      <c r="C68" s="85"/>
+      <c r="D68" s="85"/>
+      <c r="E68" s="85"/>
+      <c r="F68" s="85"/>
+      <c r="G68" s="85"/>
+      <c r="H68" s="85"/>
+      <c r="I68" s="85"/>
+      <c r="J68" s="85"/>
+      <c r="K68" s="85"/>
+      <c r="L68" s="85"/>
+      <c r="M68" s="85"/>
+      <c r="N68" s="85"/>
+      <c r="O68" s="85"/>
+      <c r="P68" s="85"/>
+      <c r="Q68" s="85"/>
       <c r="R68" s="7"/>
       <c r="S68" s="7"/>
       <c r="T68" s="7"/>
@@ -5990,11 +5994,26 @@
     </row>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="A50:C50"/>
-    <mergeCell ref="A45:C45"/>
-    <mergeCell ref="A46:C46"/>
-    <mergeCell ref="S65:Y65"/>
-    <mergeCell ref="B65:Q66"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="A53:E53"/>
+    <mergeCell ref="A33:E33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A37:C37"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="A41:E41"/>
+    <mergeCell ref="A43:C43"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A51:C51"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A28:C28"/>
     <mergeCell ref="B67:Q68"/>
     <mergeCell ref="S63:W63"/>
     <mergeCell ref="M2:Q2"/>
@@ -6011,26 +6030,11 @@
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="A58:C58"/>
     <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="A53:E53"/>
-    <mergeCell ref="A33:E33"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A37:C37"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="A41:E41"/>
-    <mergeCell ref="A43:C43"/>
-    <mergeCell ref="A26:C26"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="A51:C51"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="A50:C50"/>
+    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="A46:C46"/>
+    <mergeCell ref="S65:Y65"/>
+    <mergeCell ref="B65:Q66"/>
   </mergeCells>
   <conditionalFormatting sqref="D62:Q62">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">

</xml_diff>